<commit_message>
Release v1.0 stable: group-marker architecture, formula caching fix, validation and regression tests
</commit_message>
<xml_diff>
--- a/tests/fixtures/master_2026.xlsx
+++ b/tests/fixtures/master_2026.xlsx
@@ -17455,7 +17455,11 @@
       <c r="AO3" s="320"/>
       <c r="AP3" s="218"/>
       <c r="AQ3" s="219"/>
-      <c r="AR3" s="525"/>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>Track 1-Secured</t>
+        </is>
+      </c>
       <c r="AS3" s="525"/>
       <c r="AU3" s="534"/>
       <c r="AV3" s="534"/>
@@ -26220,7 +26224,11 @@
       </c>
       <c r="AP60" s="340"/>
       <c r="AQ60" s="341"/>
-      <c r="AR60" s="525"/>
+      <c r="AR60" t="inlineStr">
+        <is>
+          <t>Track 2-Secured</t>
+        </is>
+      </c>
       <c r="AS60" s="525"/>
       <c r="AU60" s="534"/>
       <c r="AV60" s="534"/>
@@ -26516,7 +26524,11 @@
       <c r="AO67" s="495"/>
       <c r="AP67" s="496"/>
       <c r="AQ67" s="493"/>
-      <c r="AR67" s="525"/>
+      <c r="AR67" t="inlineStr">
+        <is>
+          <t>Track 1-Projections</t>
+        </is>
+      </c>
       <c r="AS67" s="525"/>
       <c r="AT67"/>
       <c r="AU67" s="534"/>
@@ -27495,7 +27507,11 @@
       <c r="AO75" s="339"/>
       <c r="AP75" s="340"/>
       <c r="AQ75" s="341"/>
-      <c r="AR75" s="525"/>
+      <c r="AR75" t="inlineStr">
+        <is>
+          <t>Track 2-Projections</t>
+        </is>
+      </c>
       <c r="AS75" s="525"/>
       <c r="AU75" s="534"/>
       <c r="AV75" s="534"/>
@@ -30553,7 +30569,11 @@
       <c r="AO105" s="334"/>
       <c r="AP105" s="295"/>
       <c r="AQ105" s="296"/>
-      <c r="AR105" s="525"/>
+      <c r="AR105" t="inlineStr">
+        <is>
+          <t>Staffing-Secured</t>
+        </is>
+      </c>
       <c r="AS105" s="525"/>
       <c r="AU105" s="534"/>
       <c r="AV105" s="534"/>

</xml_diff>